<commit_message>
Update Pareto 80/20 analysis scripts and EDA notebook results
</commit_message>
<xml_diff>
--- a/eda/ipynb/yumi/category_top5_with_names.xlsx
+++ b/eda/ipynb/yumi/category_top5_with_names.xlsx
@@ -487,31 +487,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>택배선물세트</t>
+          <t>모듬안주</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>152000</v>
+        <v>3109532</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>죽력고32도700ml</t>
+          <t>정화)사각모듬안주109g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>냉장주스(대)</t>
+          <t>꿀</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -521,45 +521,45 @@
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>51847177</v>
+        <v>1371975</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>칠성)콜드오렌지900ml</t>
+          <t>꽃샘)야생화꿀300g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>모듬안주</t>
+          <t>빅바이트</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>3109532</v>
+        <v>2200</v>
       </c>
       <c r="E5" t="n">
         <v>100</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>정화)사각모듬안주109g</t>
+          <t>존슨빌)폴리쉬소시지108g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>꿀</t>
+          <t>버터</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -569,69 +569,69 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>1371975</v>
+        <v>910020</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>꽃샘)야생화꿀300g</t>
+          <t>동원)모닝버터해바리기유200g</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>빅바이트</t>
+          <t>모닝빵샌드</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>2200</v>
+        <v>2900</v>
       </c>
       <c r="E7" t="n">
         <v>100</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>존슨빌)폴리쉬소시지108g</t>
+          <t>롯데)소프트에그롤</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>버터</t>
+          <t>택배선물세트</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" t="n">
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>910020</v>
+        <v>152000</v>
       </c>
       <c r="E8" t="n">
         <v>100</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>동원)모닝버터해바리기유200g</t>
+          <t>죽력고32도700ml</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>모닝빵샌드</t>
+          <t>냉장주스(대)</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -641,14 +641,14 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>2900</v>
+        <v>51847177</v>
       </c>
       <c r="E9" t="n">
         <v>100</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>롯데)소프트에그롤</t>
+          <t>칠성)콜드오렌지900ml</t>
         </is>
       </c>
     </row>

</xml_diff>